<commit_message>
Standardize normal distribution exercise.
</commit_message>
<xml_diff>
--- a/resources/Part_3_Statistics/S17_L99/3.4.Standard-normal-distribution-exercise.xlsx
+++ b/resources/Part_3_Statistics/S17_L99/3.4.Standard-normal-distribution-exercise.xlsx
@@ -1,21 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20730"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iliya Valchanov\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\D\GitRepos\StatisticsBAandDS\DataScienceBootcamp\resources\Part_3_Statistics\S17_L99\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2A32AEF-2398-4984-A90F-3CFB12AF6206}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060"/>
   </bookViews>
   <sheets>
     <sheet name="Standard normal" sheetId="3" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">'Standard normal'!$B$11:$B$90</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">'Standard normal'!$H$11:$H$90</definedName>
+  </definedNames>
+  <calcPr calcId="162913"/>
   <fileRecoveryPr autoRecover="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -26,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t>Standard normal distribution</t>
   </si>
@@ -57,11 +60,23 @@
   <si>
     <t>Original dataset</t>
   </si>
+  <si>
+    <t>Mean:</t>
+  </si>
+  <si>
+    <t>Standard Dev</t>
+  </si>
+  <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>Mean =</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -169,6 +184,1222 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.0</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:rich>
+          <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES"/>
+              <a:t>Datos originales</a:t>
+            </a:r>
+          </a:p>
+        </cx:rich>
+      </cx:tx>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="clusteredColumn" uniqueId="{7153A968-7241-4C8E-BC20-2EA13131E604}">
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:binning intervalClosed="r">
+              <cx:binCount val="20"/>
+            </cx:binning>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0"/>
+        <cx:tickLabels/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+  <cx:clrMapOvr bg1="lt1" tx1="dk1" bg2="lt2" tx2="dk2" accent1="accent1" accent2="accent2" accent3="accent3" accent4="accent4" accent5="accent5" accent6="accent6" hlink="hlink" folHlink="folHlink"/>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/chartEx2.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.1</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:rich>
+          <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES"/>
+              <a:t>Normalizado</a:t>
+            </a:r>
+          </a:p>
+        </cx:rich>
+      </cx:tx>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="clusteredColumn" uniqueId="{B2169093-1AFE-4BD4-8CE7-06D599D2CB4E}">
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:binning intervalClosed="r">
+              <cx:binCount val="20"/>
+            </cx:binning>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0"/>
+        <cx:tickLabels/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+            <a:lumOff val="10000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+            <a:lumOff val="10000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>752475</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>100012</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>238125</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>100012</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="2" name="Gráfico 1"/>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="es-ES" sz="1100"/>
+                <a:t>Este gráfico no está disponible en su versión de Excel.
+Si edita esta forma o guarda el libro en un formato de archivo diferente, el gráfico no se podrá utilizar.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>366712</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>90487</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>214312</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>90487</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="3" name="Gráfico 2"/>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="es-ES" sz="1100"/>
+                <a:t>Este gráfico no está disponible en su versión de Excel.
+Si edita esta forma o guarda el libro en un formato de archivo diferente, el gráfico no se podrá utilizar.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -467,25 +1698,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:T90"/>
-  <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" style="1"/>
-    <col min="4" max="4" width="8.88671875" style="7"/>
-    <col min="5" max="5" width="4.77734375" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="4.77734375" style="7" customWidth="1"/>
-    <col min="8" max="8" width="8.88671875" style="7"/>
-    <col min="9" max="9" width="12.109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="10" max="14" width="8.88671875" style="7"/>
+    <col min="2" max="2" width="13.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" style="1"/>
+    <col min="4" max="4" width="11.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="4.7109375" style="7" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" style="7"/>
+    <col min="9" max="9" width="12.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="10" max="14" width="8.85546875" style="7"/>
     <col min="15" max="15" width="11" style="7" bestFit="1" customWidth="1"/>
-    <col min="16" max="20" width="8.88671875" style="7"/>
-    <col min="21" max="16384" width="8.88671875" style="1"/>
+    <col min="16" max="20" width="8.85546875" style="7"/>
+    <col min="21" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:20" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
@@ -526,7 +1757,7 @@
       <c r="S2" s="1"/>
       <c r="T2" s="1"/>
     </row>
-    <row r="3" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
@@ -551,7 +1782,7 @@
       <c r="S3" s="1"/>
       <c r="T3" s="1"/>
     </row>
-    <row r="4" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>2</v>
       </c>
@@ -576,7 +1807,7 @@
       <c r="S4" s="1"/>
       <c r="T4" s="1"/>
     </row>
-    <row r="5" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>3</v>
       </c>
@@ -601,7 +1832,7 @@
       <c r="S5" s="1"/>
       <c r="T5" s="1"/>
     </row>
-    <row r="6" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
@@ -626,7 +1857,7 @@
       <c r="S6" s="1"/>
       <c r="T6" s="1"/>
     </row>
-    <row r="7" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B7" s="5"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -646,7 +1877,7 @@
       <c r="S7" s="1"/>
       <c r="T7" s="1"/>
     </row>
-    <row r="8" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B8" s="5"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -666,11 +1897,27 @@
       <c r="S8" s="1"/>
       <c r="T8" s="1"/>
     </row>
-    <row r="10" spans="2:20" ht="12.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:20" ht="12.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I10" s="4"/>
+      <c r="C10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="9">
+        <f>SUM(B11:B90)/COUNT(B11:B90)</f>
+        <v>743.02708333333317</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="J10" s="9">
+        <f>SUM(H11:H90)/COUNT(H11:H90)</f>
+        <v>2.6423307986078726E-15</v>
+      </c>
       <c r="N10" s="8"/>
       <c r="O10" s="4"/>
     </row>
@@ -678,15 +1925,36 @@
       <c r="B11" s="10">
         <v>567.45000000000005</v>
       </c>
-      <c r="I11" s="9"/>
+      <c r="C11" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="7">
+        <f>_xlfn.STDEV.S(B11:B90)</f>
+        <v>73.953060547763371</v>
+      </c>
+      <c r="H11" s="7">
+        <f>(B11-$D$10)/$D$11</f>
+        <v>-2.3741692640284278</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="J11" s="7">
+        <f>_xlfn.STDEV.S(H11:H90)</f>
+        <v>0.99999999999999967</v>
+      </c>
       <c r="O11" s="9"/>
     </row>
-    <row r="12" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B12" s="10">
         <v>572.45000000000005</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="4"/>
+      <c r="H12" s="7">
+        <f t="shared" ref="H12:H75" si="0">(B12-$D$10)/$D$11</f>
+        <v>-2.3065588100057615</v>
+      </c>
       <c r="I12" s="9"/>
       <c r="K12" s="4"/>
       <c r="L12" s="9"/>
@@ -695,7 +1963,7 @@
       <c r="Q12" s="4"/>
       <c r="R12" s="9"/>
     </row>
-    <row r="13" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B13" s="10">
         <v>572.45000000000005</v>
       </c>
@@ -703,6 +1971,10 @@
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
       <c r="G13" s="9"/>
+      <c r="H13" s="7">
+        <f t="shared" si="0"/>
+        <v>-2.3065588100057615</v>
+      </c>
       <c r="I13" s="9"/>
       <c r="K13" s="4"/>
       <c r="L13" s="9"/>
@@ -715,14 +1987,22 @@
       <c r="B14" s="10">
         <v>589.11666666666679</v>
       </c>
+      <c r="H14" s="7">
+        <f t="shared" si="0"/>
+        <v>-2.081190629930207</v>
+      </c>
       <c r="I14" s="9"/>
       <c r="O14" s="9"/>
     </row>
-    <row r="15" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B15" s="10">
         <v>613.86666666666679</v>
       </c>
       <c r="C15" s="6"/>
+      <c r="H15" s="7">
+        <f t="shared" si="0"/>
+        <v>-1.7465188825180096</v>
+      </c>
       <c r="I15" s="9"/>
       <c r="J15" s="4"/>
       <c r="O15" s="9"/>
@@ -732,6 +2012,10 @@
       <c r="B16" s="10">
         <v>615.7833333333333</v>
       </c>
+      <c r="H16" s="7">
+        <f t="shared" si="0"/>
+        <v>-1.7206015418093228</v>
+      </c>
       <c r="I16" s="9"/>
       <c r="O16" s="9"/>
     </row>
@@ -739,6 +2023,10 @@
       <c r="B17" s="10">
         <v>628.45000000000005</v>
       </c>
+      <c r="H17" s="7">
+        <f t="shared" si="0"/>
+        <v>-1.5493217249519009</v>
+      </c>
       <c r="I17" s="9"/>
       <c r="O17" s="9"/>
     </row>
@@ -746,6 +2034,10 @@
       <c r="B18" s="10">
         <v>644.86666666666679</v>
       </c>
+      <c r="H18" s="7">
+        <f t="shared" si="0"/>
+        <v>-1.3273340675774794</v>
+      </c>
       <c r="I18" s="9"/>
       <c r="O18" s="9"/>
     </row>
@@ -753,6 +2045,10 @@
       <c r="B19" s="10">
         <v>650.45000000000005</v>
       </c>
+      <c r="H19" s="7">
+        <f t="shared" si="0"/>
+        <v>-1.2518357272521701</v>
+      </c>
       <c r="I19" s="9"/>
       <c r="O19" s="9"/>
     </row>
@@ -760,6 +2056,10 @@
       <c r="B20" s="10">
         <v>652.20000000000005</v>
       </c>
+      <c r="H20" s="7">
+        <f t="shared" si="0"/>
+        <v>-1.2281720683442368</v>
+      </c>
       <c r="I20" s="9"/>
       <c r="O20" s="9"/>
     </row>
@@ -767,6 +2067,10 @@
       <c r="B21" s="10">
         <v>656.86666666666679</v>
       </c>
+      <c r="H21" s="7">
+        <f t="shared" si="0"/>
+        <v>-1.1650689779230807</v>
+      </c>
       <c r="I21" s="9"/>
       <c r="O21" s="9"/>
     </row>
@@ -774,6 +2078,10 @@
       <c r="B22" s="10">
         <v>661.45</v>
       </c>
+      <c r="H22" s="7">
+        <f t="shared" si="0"/>
+        <v>-1.1030927284023044</v>
+      </c>
       <c r="I22" s="9"/>
       <c r="O22" s="9"/>
     </row>
@@ -781,6 +2089,10 @@
       <c r="B23" s="10">
         <v>666.45</v>
       </c>
+      <c r="H23" s="7">
+        <f t="shared" si="0"/>
+        <v>-1.0354822743796384</v>
+      </c>
       <c r="I23" s="9"/>
       <c r="O23" s="9"/>
     </row>
@@ -788,6 +2100,10 @@
       <c r="B24" s="10">
         <v>667.7</v>
       </c>
+      <c r="H24" s="7">
+        <f t="shared" si="0"/>
+        <v>-1.0185796608739719</v>
+      </c>
       <c r="I24" s="9"/>
       <c r="O24" s="9"/>
     </row>
@@ -795,6 +2111,10 @@
       <c r="B25" s="10">
         <v>668.95</v>
       </c>
+      <c r="H25" s="7">
+        <f t="shared" si="0"/>
+        <v>-1.0016770473683052</v>
+      </c>
       <c r="I25" s="9"/>
       <c r="O25" s="9"/>
     </row>
@@ -802,6 +2122,10 @@
       <c r="B26" s="10">
         <v>675.2833333333333</v>
       </c>
+      <c r="H26" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.91603713893959593</v>
+      </c>
       <c r="I26" s="9"/>
       <c r="O26" s="9"/>
     </row>
@@ -809,6 +2133,10 @@
       <c r="B27" s="10">
         <v>675.7833333333333</v>
       </c>
+      <c r="H27" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.9092760935373293</v>
+      </c>
       <c r="I27" s="9"/>
       <c r="O27" s="9"/>
     </row>
@@ -816,6 +2144,10 @@
       <c r="B28" s="10">
         <v>685.5333333333333</v>
       </c>
+      <c r="H28" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.77743570819313035</v>
+      </c>
       <c r="I28" s="9"/>
       <c r="O28" s="9"/>
     </row>
@@ -823,6 +2155,10 @@
       <c r="B29" s="10">
         <v>694.2833333333333</v>
       </c>
+      <c r="H29" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.65911741365346466</v>
+      </c>
       <c r="I29" s="9"/>
       <c r="O29" s="9"/>
     </row>
@@ -830,6 +2166,10 @@
       <c r="B30" s="10">
         <v>697.61666666666679</v>
       </c>
+      <c r="H30" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.61404377763835183</v>
+      </c>
       <c r="I30" s="9"/>
       <c r="O30" s="9"/>
     </row>
@@ -837,6 +2177,10 @@
       <c r="B31" s="10">
         <v>705.7833333333333</v>
       </c>
+      <c r="H31" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.5036133694013325</v>
+      </c>
       <c r="I31" s="9"/>
       <c r="O31" s="9"/>
     </row>
@@ -844,6 +2188,10 @@
       <c r="B32" s="10">
         <v>705.86666666666679</v>
       </c>
+      <c r="H32" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.50248652850095266</v>
+      </c>
       <c r="I32" s="9"/>
       <c r="O32" s="9"/>
     </row>
@@ -851,6 +2199,10 @@
       <c r="B33" s="10">
         <v>708.11666666666679</v>
       </c>
+      <c r="H33" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.47206182419075293</v>
+      </c>
       <c r="I33" s="9"/>
       <c r="O33" s="9"/>
     </row>
@@ -858,6 +2210,10 @@
       <c r="B34" s="10">
         <v>711.0333333333333</v>
       </c>
+      <c r="H34" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.43262239267753305</v>
+      </c>
       <c r="I34" s="9"/>
       <c r="O34" s="9"/>
     </row>
@@ -865,6 +2221,10 @@
       <c r="B35" s="10">
         <v>714.0333333333333</v>
       </c>
+      <c r="H35" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.39205612026393338</v>
+      </c>
       <c r="I35" s="9"/>
       <c r="O35" s="9"/>
     </row>
@@ -872,6 +2232,10 @@
       <c r="B36" s="10">
         <v>716.0333333333333</v>
       </c>
+      <c r="H36" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.36501193865486692</v>
+      </c>
       <c r="I36" s="9"/>
       <c r="O36" s="9"/>
     </row>
@@ -879,6 +2243,10 @@
       <c r="B37" s="10">
         <v>722.2833333333333</v>
       </c>
+      <c r="H37" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.28049887112653427</v>
+      </c>
       <c r="I37" s="9"/>
       <c r="O37" s="9"/>
     </row>
@@ -886,6 +2254,10 @@
       <c r="B38" s="10">
         <v>728.11666666666679</v>
       </c>
+      <c r="H38" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.2016200081000884</v>
+      </c>
       <c r="I38" s="9"/>
       <c r="O38" s="9"/>
     </row>
@@ -893,6 +2265,10 @@
       <c r="B39" s="10">
         <v>728.7</v>
       </c>
+      <c r="H39" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.19373212179744503</v>
+      </c>
       <c r="I39" s="9"/>
       <c r="O39" s="9"/>
     </row>
@@ -900,6 +2276,10 @@
       <c r="B40" s="10">
         <v>729.0333333333333</v>
       </c>
+      <c r="H40" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.18922475819593498</v>
+      </c>
       <c r="I40" s="9"/>
       <c r="O40" s="9"/>
     </row>
@@ -907,6 +2287,10 @@
       <c r="B41" s="10">
         <v>730.11666666666679</v>
       </c>
+      <c r="H41" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.17457582649102193</v>
+      </c>
       <c r="I41" s="9"/>
       <c r="O41" s="9"/>
     </row>
@@ -914,6 +2298,10 @@
       <c r="B42" s="10">
         <v>731.95</v>
       </c>
+      <c r="H42" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.14978532668271205</v>
+      </c>
       <c r="I42" s="9"/>
       <c r="O42" s="9"/>
     </row>
@@ -921,6 +2309,10 @@
       <c r="B43" s="10">
         <v>735.0333333333333</v>
       </c>
+      <c r="H43" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.10809221336873563</v>
+      </c>
       <c r="I43" s="9"/>
       <c r="O43" s="9"/>
     </row>
@@ -928,6 +2320,10 @@
       <c r="B44" s="10">
         <v>736.95</v>
       </c>
+      <c r="H44" s="7">
+        <f t="shared" si="0"/>
+        <v>-8.2174872660045931E-2</v>
+      </c>
       <c r="I44" s="9"/>
       <c r="O44" s="9"/>
     </row>
@@ -935,6 +2331,10 @@
       <c r="B45" s="10">
         <v>737.36666666666679</v>
       </c>
+      <c r="H45" s="7">
+        <f t="shared" si="0"/>
+        <v>-7.654066815815605E-2</v>
+      </c>
       <c r="I45" s="9"/>
       <c r="O45" s="9"/>
     </row>
@@ -942,6 +2342,10 @@
       <c r="B46" s="10">
         <v>738.2833333333333</v>
       </c>
+      <c r="H46" s="7">
+        <f t="shared" si="0"/>
+        <v>-6.4145418254002648E-2</v>
+      </c>
       <c r="I46" s="9"/>
       <c r="O46" s="9"/>
     </row>
@@ -949,6 +2353,10 @@
       <c r="B47" s="10">
         <v>739.7833333333333</v>
       </c>
+      <c r="H47" s="7">
+        <f t="shared" si="0"/>
+        <v>-4.3862282047202807E-2</v>
+      </c>
       <c r="I47" s="9"/>
       <c r="O47" s="9"/>
     </row>
@@ -956,6 +2364,10 @@
       <c r="B48" s="10">
         <v>740.61666666666679</v>
       </c>
+      <c r="H48" s="7">
+        <f t="shared" si="0"/>
+        <v>-3.2593873043423073E-2</v>
+      </c>
       <c r="I48" s="9"/>
       <c r="O48" s="9"/>
     </row>
@@ -963,6 +2375,10 @@
       <c r="B49" s="10">
         <v>743.61666666666679</v>
       </c>
+      <c r="H49" s="7">
+        <f t="shared" si="0"/>
+        <v>7.9723993701766097E-3</v>
+      </c>
       <c r="I49" s="9"/>
       <c r="O49" s="9"/>
     </row>
@@ -970,6 +2386,10 @@
       <c r="B50" s="10">
         <v>747.2</v>
       </c>
+      <c r="H50" s="7">
+        <f t="shared" si="0"/>
+        <v>5.6426558086419644E-2</v>
+      </c>
       <c r="I50" s="9"/>
       <c r="O50" s="9"/>
     </row>
@@ -977,6 +2397,10 @@
       <c r="B51" s="10">
         <v>748.2</v>
       </c>
+      <c r="H51" s="7">
+        <f t="shared" si="0"/>
+        <v>6.9948648890952869E-2</v>
+      </c>
       <c r="I51" s="9"/>
       <c r="O51" s="9"/>
     </row>
@@ -984,6 +2408,10 @@
       <c r="B52" s="10">
         <v>748.2833333333333</v>
       </c>
+      <c r="H52" s="7">
+        <f t="shared" si="0"/>
+        <v>7.1075489791329619E-2</v>
+      </c>
       <c r="I52" s="9"/>
       <c r="O52" s="9"/>
     </row>
@@ -991,6 +2419,10 @@
       <c r="B53" s="10">
         <v>748.5333333333333</v>
       </c>
+      <c r="H53" s="7">
+        <f t="shared" si="0"/>
+        <v>7.445601249246292E-2</v>
+      </c>
       <c r="I53" s="9"/>
       <c r="O53" s="9"/>
     </row>
@@ -998,6 +2430,10 @@
       <c r="B54" s="10">
         <v>750.0333333333333</v>
       </c>
+      <c r="H54" s="7">
+        <f t="shared" si="0"/>
+        <v>9.4739148699262768E-2</v>
+      </c>
       <c r="I54" s="9"/>
       <c r="O54" s="9"/>
     </row>
@@ -1005,6 +2441,10 @@
       <c r="B55" s="10">
         <v>752.11666666666679</v>
       </c>
+      <c r="H55" s="7">
+        <f t="shared" si="0"/>
+        <v>0.12291017120870903</v>
+      </c>
       <c r="I55" s="9"/>
       <c r="O55" s="9"/>
     </row>
@@ -1012,6 +2452,10 @@
       <c r="B56" s="10">
         <v>754.7</v>
       </c>
+      <c r="H56" s="7">
+        <f t="shared" si="0"/>
+        <v>0.15784223912041884</v>
+      </c>
       <c r="I56" s="9"/>
       <c r="O56" s="9"/>
     </row>
@@ -1019,6 +2463,10 @@
       <c r="B57" s="10">
         <v>755.0333333333333</v>
       </c>
+      <c r="H57" s="7">
+        <f t="shared" si="0"/>
+        <v>0.16234960272192889</v>
+      </c>
       <c r="I57" s="9"/>
       <c r="O57" s="9"/>
     </row>
@@ -1026,6 +2474,10 @@
       <c r="B58" s="10">
         <v>758.36666666666667</v>
       </c>
+      <c r="H58" s="7">
+        <f t="shared" si="0"/>
+        <v>0.20742323873704016</v>
+      </c>
       <c r="I58" s="9"/>
       <c r="O58" s="9"/>
     </row>
@@ -1033,6 +2485,10 @@
       <c r="B59" s="10">
         <v>760.53333333333342</v>
       </c>
+      <c r="H59" s="7">
+        <f t="shared" si="0"/>
+        <v>0.23672110214686318</v>
+      </c>
       <c r="I59" s="9"/>
       <c r="O59" s="9"/>
     </row>
@@ -1040,6 +2496,10 @@
       <c r="B60" s="10">
         <v>764.03333333333342</v>
       </c>
+      <c r="H60" s="7">
+        <f t="shared" si="0"/>
+        <v>0.28404841996272945</v>
+      </c>
       <c r="I60" s="9"/>
       <c r="O60" s="9"/>
     </row>
@@ -1047,6 +2507,10 @@
       <c r="B61" s="10">
         <v>769.28333333333342</v>
       </c>
+      <c r="H61" s="7">
+        <f t="shared" si="0"/>
+        <v>0.3550393966865289</v>
+      </c>
       <c r="I61" s="9"/>
       <c r="O61" s="9"/>
     </row>
@@ -1054,6 +2518,10 @@
       <c r="B62" s="10">
         <v>775.45</v>
       </c>
+      <c r="H62" s="7">
+        <f t="shared" si="0"/>
+        <v>0.43842562331448326</v>
+      </c>
       <c r="I62" s="9"/>
       <c r="O62" s="9"/>
     </row>
@@ -1061,6 +2529,10 @@
       <c r="B63" s="10">
         <v>781.2</v>
       </c>
+      <c r="H63" s="7">
+        <f t="shared" si="0"/>
+        <v>0.51617764544054934</v>
+      </c>
       <c r="I63" s="9"/>
       <c r="O63" s="9"/>
     </row>
@@ -1068,6 +2540,10 @@
       <c r="B64" s="10">
         <v>781.7</v>
       </c>
+      <c r="H64" s="7">
+        <f t="shared" si="0"/>
+        <v>0.52293869084281597</v>
+      </c>
       <c r="I64" s="9"/>
       <c r="O64" s="9"/>
     </row>
@@ -1075,6 +2551,10 @@
       <c r="B65" s="10">
         <v>785.61666666666667</v>
       </c>
+      <c r="H65" s="7">
+        <f t="shared" si="0"/>
+        <v>0.57590021316057061</v>
+      </c>
       <c r="I65" s="9"/>
       <c r="O65" s="9"/>
     </row>
@@ -1082,6 +2562,10 @@
       <c r="B66" s="10">
         <v>792.78333333333342</v>
       </c>
+      <c r="H66" s="7">
+        <f t="shared" si="0"/>
+        <v>0.67280853059305967</v>
+      </c>
       <c r="I66" s="9"/>
       <c r="O66" s="9"/>
     </row>
@@ -1089,6 +2573,10 @@
       <c r="B67" s="10">
         <v>793.36666666666667</v>
       </c>
+      <c r="H67" s="7">
+        <f t="shared" si="0"/>
+        <v>0.68069641689570304</v>
+      </c>
       <c r="I67" s="9"/>
       <c r="O67" s="9"/>
     </row>
@@ -1096,6 +2584,10 @@
       <c r="B68" s="10">
         <v>795.28333333333342</v>
       </c>
+      <c r="H68" s="7">
+        <f t="shared" si="0"/>
+        <v>0.70661375760439282</v>
+      </c>
       <c r="I68" s="9"/>
       <c r="O68" s="9"/>
     </row>
@@ -1103,6 +2595,10 @@
       <c r="B69" s="10">
         <v>797.61666666666667</v>
       </c>
+      <c r="H69" s="7">
+        <f t="shared" si="0"/>
+        <v>0.73816530281496928</v>
+      </c>
       <c r="I69" s="9"/>
       <c r="O69" s="9"/>
     </row>
@@ -1110,6 +2606,10 @@
       <c r="B70" s="10">
         <v>798.95</v>
       </c>
+      <c r="H70" s="7">
+        <f t="shared" si="0"/>
+        <v>0.75619475722101415</v>
+      </c>
       <c r="I70" s="9"/>
       <c r="O70" s="9"/>
     </row>
@@ -1117,6 +2617,10 @@
       <c r="B71" s="10">
         <v>799.7</v>
       </c>
+      <c r="H71" s="7">
+        <f t="shared" si="0"/>
+        <v>0.76633632532441398</v>
+      </c>
       <c r="I71" s="9"/>
       <c r="O71" s="9"/>
     </row>
@@ -1124,6 +2628,10 @@
       <c r="B72" s="10">
         <v>799.95</v>
       </c>
+      <c r="H72" s="7">
+        <f t="shared" si="0"/>
+        <v>0.7697168480255473</v>
+      </c>
       <c r="I72" s="9"/>
       <c r="O72" s="9"/>
     </row>
@@ -1131,6 +2639,10 @@
       <c r="B73" s="10">
         <v>810.86666666666667</v>
       </c>
+      <c r="H73" s="7">
+        <f t="shared" si="0"/>
+        <v>0.91733300597503453</v>
+      </c>
       <c r="I73" s="9"/>
       <c r="O73" s="9"/>
     </row>
@@ -1138,6 +2650,10 @@
       <c r="B74" s="10">
         <v>811.53333333333342</v>
       </c>
+      <c r="H74" s="7">
+        <f t="shared" si="0"/>
+        <v>0.92634773317805774</v>
+      </c>
       <c r="I74" s="9"/>
       <c r="O74" s="9"/>
     </row>
@@ -1145,6 +2661,10 @@
       <c r="B75" s="10">
         <v>813.61666666666667</v>
       </c>
+      <c r="H75" s="7">
+        <f t="shared" si="0"/>
+        <v>0.95451875568750089</v>
+      </c>
       <c r="I75" s="9"/>
       <c r="O75" s="9"/>
     </row>
@@ -1152,6 +2672,10 @@
       <c r="B76" s="10">
         <v>814.03333333333342</v>
       </c>
+      <c r="H76" s="7">
+        <f t="shared" ref="H76:H90" si="1">(B76-$D$10)/$D$11</f>
+        <v>0.96015296018939078</v>
+      </c>
       <c r="I76" s="9"/>
       <c r="O76" s="9"/>
     </row>
@@ -1159,6 +2683,10 @@
       <c r="B77" s="10">
         <v>814.78333333333342</v>
       </c>
+      <c r="H77" s="7">
+        <f t="shared" si="1"/>
+        <v>0.97029452829279073</v>
+      </c>
       <c r="I77" s="9"/>
       <c r="O77" s="9"/>
     </row>
@@ -1166,6 +2694,10 @@
       <c r="B78" s="10">
         <v>817.86666666666667</v>
       </c>
+      <c r="H78" s="7">
+        <f t="shared" si="1"/>
+        <v>1.011987641606767</v>
+      </c>
       <c r="I78" s="9"/>
       <c r="O78" s="9"/>
     </row>
@@ -1173,6 +2705,10 @@
       <c r="B79" s="10">
         <v>818.86666666666667</v>
       </c>
+      <c r="H79" s="7">
+        <f t="shared" si="1"/>
+        <v>1.0255097324113003</v>
+      </c>
       <c r="I79" s="9"/>
       <c r="O79" s="9"/>
     </row>
@@ -1180,6 +2716,10 @@
       <c r="B80" s="10">
         <v>820.7</v>
       </c>
+      <c r="H80" s="7">
+        <f t="shared" si="1"/>
+        <v>1.0503002322196118</v>
+      </c>
       <c r="I80" s="9"/>
       <c r="O80" s="9"/>
     </row>
@@ -1187,6 +2727,10 @@
       <c r="B81" s="10">
         <v>821.11666666666667</v>
       </c>
+      <c r="H81" s="7">
+        <f t="shared" si="1"/>
+        <v>1.0559344367215</v>
+      </c>
       <c r="I81" s="9"/>
       <c r="O81" s="9"/>
     </row>
@@ -1194,6 +2738,10 @@
       <c r="B82" s="10">
         <v>825.61666666666667</v>
       </c>
+      <c r="H82" s="7">
+        <f t="shared" si="1"/>
+        <v>1.1167838453418997</v>
+      </c>
       <c r="I82" s="9"/>
       <c r="O82" s="9"/>
     </row>
@@ -1201,6 +2749,10 @@
       <c r="B83" s="10">
         <v>828.61666666666667</v>
       </c>
+      <c r="H83" s="7">
+        <f t="shared" si="1"/>
+        <v>1.1573501177554992</v>
+      </c>
       <c r="I83" s="9"/>
       <c r="O83" s="9"/>
     </row>
@@ -1208,6 +2760,10 @@
       <c r="B84" s="10">
         <v>841.45</v>
       </c>
+      <c r="H84" s="7">
+        <f t="shared" si="1"/>
+        <v>1.3308836164136761</v>
+      </c>
       <c r="I84" s="9"/>
       <c r="O84" s="9"/>
     </row>
@@ -1215,6 +2771,10 @@
       <c r="B85" s="10">
         <v>842.03333333333342</v>
       </c>
+      <c r="H85" s="7">
+        <f t="shared" si="1"/>
+        <v>1.3387715027163212</v>
+      </c>
       <c r="I85" s="9"/>
       <c r="O85" s="9"/>
     </row>
@@ -1222,6 +2782,10 @@
       <c r="B86" s="10">
         <v>842.86666666666667</v>
       </c>
+      <c r="H86" s="7">
+        <f t="shared" si="1"/>
+        <v>1.3500399117200979</v>
+      </c>
       <c r="I86" s="9"/>
       <c r="O86" s="9"/>
     </row>
@@ -1229,6 +2793,10 @@
       <c r="B87" s="10">
         <v>849.61666666666667</v>
       </c>
+      <c r="H87" s="7">
+        <f t="shared" si="1"/>
+        <v>1.441314024650697</v>
+      </c>
       <c r="I87" s="9"/>
       <c r="O87" s="9"/>
     </row>
@@ -1236,6 +2804,10 @@
       <c r="B88" s="10">
         <v>874.7</v>
       </c>
+      <c r="H88" s="7">
+        <f t="shared" si="1"/>
+        <v>1.780493135664406</v>
+      </c>
       <c r="I88" s="9"/>
       <c r="O88" s="9"/>
     </row>
@@ -1243,6 +2815,10 @@
       <c r="B89" s="10">
         <v>878.78333333333342</v>
       </c>
+      <c r="H89" s="7">
+        <f t="shared" si="1"/>
+        <v>1.8357083397829173</v>
+      </c>
       <c r="I89" s="9"/>
       <c r="O89" s="9"/>
     </row>
@@ -1250,11 +2826,16 @@
       <c r="B90" s="11">
         <v>897.45</v>
       </c>
+      <c r="H90" s="7">
+        <f t="shared" si="1"/>
+        <v>2.0881207014675369</v>
+      </c>
       <c r="I90" s="9"/>
       <c r="O90" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>